<commit_message>
Update Chorrillo project files and add EzImpulse
Added EzImpulse_v1.0.xlsm and new ChorrilloV1 SolidWorks part and assembly files. Updated and replaced several SLDPRT and SLDASM files, removing older versions. Updated PFlammam - Chorrillo.xlsm and o-ring_2.4.xlsx with new changes.
</commit_message>
<xml_diff>
--- a/PFlammam - Chorrillo rev 1/o-ring_2.4.xlsx
+++ b/PFlammam - Chorrillo rev 1/o-ring_2.4.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Engineering\01 Repos\The-thermal-repository\PFlammam - Lucia V1 rev3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Engineering\01 Repos\The-thermal-repository\PFlammam - Chorrillo rev 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E4F522-5A04-4A34-A9F8-A2F0CC85B7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C1B0EFD-9374-4B22-A077-C2C2B930C003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookPassword="C7BC" lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="1910" yWindow="1340" windowWidth="14400" windowHeight="8180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="-010" sheetId="1" r:id="rId1"/>
@@ -68,7 +68,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Simply enter values for casing ID and clearance. 
 Recommended o-ring size is given.
@@ -85,7 +85,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter motor casing inside diameter (inches)
 6 in. max.
@@ -100,7 +100,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter total clearance between nozzle and casing ID.
 Recommended between
@@ -117,7 +117,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Recommended o-ring size
 </t>
@@ -131,7 +131,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Should be 2% minimum, 10% maximum
 </t>
@@ -145,7 +145,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Diametrical clearance in "thou".
 Should be between 1 and 5 "thou"
@@ -170,7 +170,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Simply enter values for casing ID and clearance. 
 Recommended o-ring size is given.
@@ -187,7 +187,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter motor casing inside diameter (inches)
 </t>
@@ -201,7 +201,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter total clearance between nozzle and casing ID.
 Recommended between
@@ -218,7 +218,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Recommended o-ring size
 </t>
@@ -232,7 +232,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Should be 2% minimum, 10% maximum
 </t>
@@ -246,7 +246,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Diametrical clearance in "thou".
 Should be between 1 and 5 "thou"
@@ -271,7 +271,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Simply enter values for casing ID and clearance. 
 Recommended o-ring size is given.
@@ -288,7 +288,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter motor casing inside diameter (inches)
 </t>
@@ -302,7 +302,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Enter total clearance between nozzle and casing ID.
 Should be between
@@ -318,7 +318,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Recommended o-ring size
 </t>
@@ -332,7 +332,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Should be 2% minimum, 10% maximum
 </t>
@@ -346,7 +346,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Diametrical clearance in "thou".
 Should be between 1 and 5 "thou"
@@ -371,7 +371,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Simply enter values for casing ID and clearance. 
 Recommended o-ring size is given.
@@ -388,7 +388,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter motor casing inside diameter (inches)
 </t>
@@ -402,7 +402,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Enter total clearance between nozzle and casing ID.
 Should be between
@@ -419,7 +419,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Recommended o-ring size
 </t>
@@ -433,7 +433,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Should be 2% minimum, 10% maximum
 </t>
@@ -447,7 +447,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">Diametrical clearance in "thou".
 Should be between 1 and 5 "thou"
@@ -949,10 +949,12 @@
       <sz val="10"/>
       <color indexed="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -964,7 +966,7 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2423,45 +2425,47 @@
     </row>
     <row r="16" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="72">
-        <v>1.223622</v>
+        <f>52.5018/25.4</f>
+        <v>2.0670000000000002</v>
       </c>
       <c r="C16" s="81">
-        <v>2E-3</v>
+        <f>0.004*2</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="D16" s="83">
         <f>B16-C16</f>
-        <v>1.221622</v>
+        <v>2.0590000000000002</v>
       </c>
       <c r="E16" s="96">
         <f>VLOOKUP(($D16-2*0.051),tab2c,3)</f>
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F16" s="43">
         <f>VLOOKUP($E16,tab1c,4)</f>
-        <v>1.1909999999999998</v>
+        <v>2.004</v>
       </c>
       <c r="G16" s="36">
         <f>VLOOKUP($E16,tab1c,5)</f>
-        <v>1.1809999999999998</v>
+        <v>1.9890000000000001</v>
       </c>
       <c r="H16" s="37">
         <f>VLOOKUP($E16,tab1c,6)</f>
-        <v>1.2009999999999998</v>
+        <v>2.0190000000000001</v>
       </c>
       <c r="I16">
         <f>D16-2*0.051</f>
-        <v>1.1196219999999999</v>
+        <v>1.9570000000000001</v>
       </c>
       <c r="J16" s="38">
         <f>(I16-VLOOKUP($E16,tab1c,2))/VLOOKUP($E16,tab1c,2)</f>
-        <v>6.529210275927684E-2</v>
+        <v>4.9892703862660925E-2</v>
       </c>
     </row>
     <row r="17" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="39"/>
       <c r="C17" s="73">
         <f>C16*1000</f>
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F17" s="37"/>
     </row>
@@ -4837,47 +4841,47 @@
     </row>
     <row r="16" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="72">
-        <f>35.08/25.4</f>
-        <v>1.3811023622047245</v>
+        <f>52.5018/25.4</f>
+        <v>2.0670000000000002</v>
       </c>
       <c r="C16" s="81">
-        <f>2*0.002</f>
-        <v>4.0000000000000001E-3</v>
+        <f>0.004*2</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="D16" s="83">
         <f>B16-C16</f>
-        <v>1.3771023622047245</v>
+        <v>2.0590000000000002</v>
       </c>
       <c r="E16" s="71">
         <f>VLOOKUP(($D16-2*0.082),table2,3)</f>
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="F16" s="43">
         <f>VLOOKUP($E16,_tab1,4)</f>
-        <v>1.38</v>
+        <v>2.0049999999999999</v>
       </c>
       <c r="G16" s="36">
         <f>VLOOKUP($E16,_tab1,5)</f>
-        <v>1.3679999999999999</v>
+        <v>1.99</v>
       </c>
       <c r="H16" s="37">
         <f>VLOOKUP($E16,_tab1,6)</f>
-        <v>1.3919999999999999</v>
+        <v>2.02</v>
       </c>
       <c r="I16">
         <f>D16-2*0.082</f>
-        <v>1.2131023622047246</v>
+        <v>1.8950000000000002</v>
       </c>
       <c r="J16" s="38">
         <f>(I16-VLOOKUP($E16,_tab1,2))/VLOOKUP($E16,_tab1,2)</f>
-        <v>3.3306952474211782E-2</v>
+        <v>5.3362979433018515E-2</v>
       </c>
     </row>
     <row r="17" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="39"/>
       <c r="C17" s="73">
         <f>C16*1000</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E17" s="36"/>
       <c r="F17" s="37"/>
@@ -7652,45 +7656,47 @@
     </row>
     <row r="16" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="72">
-        <v>1.2254</v>
+        <f>52.5018/25.4</f>
+        <v>2.0670000000000002</v>
       </c>
       <c r="C16" s="81">
-        <v>3.0000000000000001E-3</v>
+        <f>0.004*2</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="D16" s="83">
         <f>B16-C16</f>
-        <v>1.2224000000000002</v>
-      </c>
-      <c r="E16" s="71" t="e">
+        <v>2.0590000000000002</v>
+      </c>
+      <c r="E16" s="71">
         <f>VLOOKUP(($D16-2*0.111),table2b,3)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F16" s="43" t="e">
+        <v>224</v>
+      </c>
+      <c r="F16" s="43">
         <f>VLOOKUP($E16,tab1b,4)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G16" s="36" t="e">
+        <v>2.012</v>
+      </c>
+      <c r="G16" s="36">
         <f>VLOOKUP($E16,tab1b,5)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H16" s="37" t="e">
+        <v>1.9970000000000001</v>
+      </c>
+      <c r="H16" s="37">
         <f>VLOOKUP($E16,tab1b,6)</f>
-        <v>#N/A</v>
+        <v>2.0270000000000001</v>
       </c>
       <c r="I16">
         <f>D16-2*0.111</f>
-        <v>1.0004000000000002</v>
-      </c>
-      <c r="J16" s="38" t="e">
+        <v>1.8370000000000002</v>
+      </c>
+      <c r="J16" s="38">
         <f>(I16-VLOOKUP($E16,tab1b,2))/VLOOKUP($E16,tab1b,2)</f>
-        <v>#N/A</v>
+        <v>5.9400230680507614E-2</v>
       </c>
     </row>
     <row r="17" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="79"/>
       <c r="C17" s="73">
         <f>C16*1000</f>
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="80"/>
@@ -10593,45 +10599,47 @@
     </row>
     <row r="16" spans="2:10" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="72">
-        <v>1.224</v>
+        <f>52.5018/25.4</f>
+        <v>2.0670000000000002</v>
       </c>
       <c r="C16" s="81">
-        <v>5.0000000000000001E-3</v>
+        <f>0.004*2</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="D16" s="83">
         <f>B16-C16</f>
-        <v>1.2190000000000001</v>
-      </c>
-      <c r="E16" s="82" t="e">
+        <v>2.0590000000000002</v>
+      </c>
+      <c r="E16" s="82">
         <f>VLOOKUP(($D16-2*0.17),table2a,3)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="F16" s="35" t="e">
+        <v>326</v>
+      </c>
+      <c r="F16" s="35">
         <f>VLOOKUP($E16,tab1a,4)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="G16" s="36" t="e">
+        <v>2.02</v>
+      </c>
+      <c r="G16" s="36">
         <f>VLOOKUP($E16,tab1a,5)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="H16" s="37" t="e">
+        <v>2.0049999999999999</v>
+      </c>
+      <c r="H16" s="37">
         <f>VLOOKUP($E16,tab1a,6)</f>
-        <v>#N/A</v>
+        <v>2.0350000000000001</v>
       </c>
       <c r="I16">
         <f>D16-2*0.17</f>
-        <v>0.879</v>
-      </c>
-      <c r="J16" s="38" t="e">
+        <v>1.7190000000000001</v>
+      </c>
+      <c r="J16" s="38">
         <f>(I16-VLOOKUP($E16,tab1a,2))/VLOOKUP($E16,tab1a,2)</f>
-        <v>#N/A</v>
+        <v>7.4374999999999997E-2</v>
       </c>
     </row>
     <row r="17" spans="2:18" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="79"/>
       <c r="C17" s="73">
         <f>C16*1000</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="80"/>

</xml_diff>